<commit_message>
test: replace dummy addresses with real Vienna landmarks for geocoding validation
</commit_message>
<xml_diff>
--- a/data/raw/building_data.xlsx
+++ b/data/raw/building_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ehska\Projects\building-data-pipeline\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D550FA2-A2AA-41FD-9898-EF3EDBB59BA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F635BAD2-A558-4A6C-8774-25546DF83666}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6768" yWindow="4032" windowWidth="13128" windowHeight="7872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="building_data" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="141">
   <si>
     <t>Building_ID</t>
   </si>
@@ -84,9 +84,6 @@
     <t>B003</t>
   </si>
   <si>
-    <t>Stephansplatz 56</t>
-  </si>
-  <si>
     <t>1010</t>
   </si>
   <si>
@@ -439,6 +436,18 @@
   </si>
   <si>
     <t>M005</t>
+  </si>
+  <si>
+    <t>Höchstädtplatz 6</t>
+  </si>
+  <si>
+    <t>Welthandelsplatz 1</t>
+  </si>
+  <si>
+    <t>Stephansplatz 3</t>
+  </si>
+  <si>
+    <t>District</t>
   </si>
 </sst>
 </file>
@@ -780,6 +789,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="18.21875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -813,10 +835,10 @@
         <v>9</v>
       </c>
       <c r="K1" t="s">
+        <v>131</v>
+      </c>
+      <c r="L1" t="s">
         <v>132</v>
-      </c>
-      <c r="L1" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
@@ -824,34 +846,34 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" t="s">
-        <v>12</v>
+        <v>137</v>
+      </c>
+      <c r="C2">
+        <v>1200</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>79</v>
       </c>
       <c r="E2" t="s">
         <v>14</v>
       </c>
       <c r="F2">
-        <v>1995</v>
+        <v>2000</v>
       </c>
       <c r="G2" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="H2">
-        <v>120</v>
+        <v>25000</v>
       </c>
       <c r="I2" t="s">
-        <v>16</v>
+        <v>140</v>
       </c>
       <c r="J2">
-        <v>17760</v>
+        <v>3500000</v>
       </c>
       <c r="K2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="L2">
         <v>50000</v>
@@ -862,34 +884,34 @@
         <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>12</v>
+        <v>138</v>
+      </c>
+      <c r="C3">
+        <v>1020</v>
       </c>
       <c r="D3" t="s">
-        <v>13</v>
+        <v>79</v>
       </c>
       <c r="E3" t="s">
         <v>14</v>
       </c>
       <c r="F3">
-        <v>1995</v>
+        <v>2013</v>
       </c>
       <c r="G3" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="H3">
-        <v>120</v>
+        <v>100000</v>
       </c>
       <c r="I3" t="s">
-        <v>16</v>
+        <v>140</v>
       </c>
       <c r="J3">
-        <v>17760</v>
+        <v>9000000</v>
       </c>
       <c r="K3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="L3">
         <v>12000</v>
@@ -900,34 +922,34 @@
         <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" t="s">
-        <v>20</v>
+        <v>139</v>
+      </c>
+      <c r="C4">
+        <v>1010</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
+        <v>79</v>
       </c>
       <c r="E4" t="s">
         <v>14</v>
       </c>
       <c r="F4">
-        <v>1995</v>
+        <v>1160</v>
       </c>
       <c r="G4" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="H4">
-        <v>250</v>
+        <v>3500</v>
       </c>
       <c r="I4" t="s">
         <v>16</v>
       </c>
       <c r="J4">
-        <v>37500</v>
+        <v>500000</v>
       </c>
       <c r="K4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="L4">
         <v>85000</v>
@@ -935,16 +957,16 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
         <v>23</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>24</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>25</v>
-      </c>
-      <c r="D5" t="s">
-        <v>26</v>
       </c>
       <c r="E5" t="s">
         <v>14</v>
@@ -953,7 +975,7 @@
         <v>2005</v>
       </c>
       <c r="G5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H5">
         <v>250</v>
@@ -965,7 +987,7 @@
         <v>38250</v>
       </c>
       <c r="K5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L5">
         <v>4000</v>
@@ -973,16 +995,16 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" t="s">
         <v>27</v>
       </c>
-      <c r="B6" t="s">
-        <v>28</v>
-      </c>
       <c r="C6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" t="s">
         <v>25</v>
-      </c>
-      <c r="D6" t="s">
-        <v>26</v>
       </c>
       <c r="E6" t="s">
         <v>14</v>
@@ -991,19 +1013,19 @@
         <v>1975</v>
       </c>
       <c r="G6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H6">
         <v>1200</v>
       </c>
       <c r="I6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J6">
         <v>140400</v>
       </c>
       <c r="K6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="L6">
         <v>1500</v>
@@ -1011,16 +1033,16 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" t="s">
         <v>30</v>
       </c>
-      <c r="B7" t="s">
-        <v>31</v>
-      </c>
       <c r="C7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" t="s">
         <v>25</v>
-      </c>
-      <c r="D7" t="s">
-        <v>26</v>
       </c>
       <c r="E7" t="s">
         <v>14</v>
@@ -1029,13 +1051,13 @@
         <v>2005</v>
       </c>
       <c r="G7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H7">
         <v>1200</v>
       </c>
       <c r="I7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J7">
         <v>181200</v>
@@ -1043,16 +1065,16 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" t="s">
         <v>33</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>34</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>35</v>
-      </c>
-      <c r="D8" t="s">
-        <v>36</v>
       </c>
       <c r="E8" t="s">
         <v>14</v>
@@ -1067,7 +1089,7 @@
         <v>2500</v>
       </c>
       <c r="I8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J8">
         <v>317500</v>
@@ -1075,16 +1097,16 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" t="s">
         <v>37</v>
       </c>
-      <c r="B9" t="s">
-        <v>38</v>
-      </c>
       <c r="C9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" t="s">
         <v>20</v>
-      </c>
-      <c r="D9" t="s">
-        <v>21</v>
       </c>
       <c r="E9" t="s">
         <v>14</v>
@@ -1093,7 +1115,7 @@
         <v>2015</v>
       </c>
       <c r="G9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H9">
         <v>1200</v>
@@ -1107,16 +1129,16 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" t="s">
         <v>39</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>40</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>41</v>
-      </c>
-      <c r="D10" t="s">
-        <v>42</v>
       </c>
       <c r="E10" t="s">
         <v>14</v>
@@ -1131,21 +1153,21 @@
         <v>800</v>
       </c>
       <c r="I10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" t="s">
         <v>43</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>44</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>45</v>
-      </c>
-      <c r="D11" t="s">
-        <v>46</v>
       </c>
       <c r="E11" t="s">
         <v>14</v>
@@ -1154,13 +1176,13 @@
         <v>1985</v>
       </c>
       <c r="G11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H11">
         <v>250</v>
       </c>
       <c r="I11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J11">
         <v>22500</v>
@@ -1168,16 +1190,16 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
+        <v>46</v>
+      </c>
+      <c r="B12" t="s">
         <v>47</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>48</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>49</v>
-      </c>
-      <c r="D12" t="s">
-        <v>50</v>
       </c>
       <c r="E12" t="s">
         <v>14</v>
@@ -1186,13 +1208,13 @@
         <v>1995</v>
       </c>
       <c r="G12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H12">
         <v>2500</v>
       </c>
       <c r="I12" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J12">
         <v>290000</v>
@@ -1200,16 +1222,16 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
+        <v>52</v>
+      </c>
+      <c r="B13" t="s">
         <v>53</v>
       </c>
-      <c r="B13" t="s">
-        <v>54</v>
-      </c>
       <c r="C13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" t="s">
         <v>20</v>
-      </c>
-      <c r="D13" t="s">
-        <v>21</v>
       </c>
       <c r="E13" t="s">
         <v>14</v>
@@ -1218,13 +1240,13 @@
         <v>2005</v>
       </c>
       <c r="G13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H13">
         <v>250</v>
       </c>
       <c r="I13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J13">
         <v>24750</v>
@@ -1232,16 +1254,16 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
+        <v>54</v>
+      </c>
+      <c r="B14" t="s">
         <v>55</v>
       </c>
-      <c r="B14" t="s">
-        <v>56</v>
-      </c>
       <c r="C14" t="s">
+        <v>44</v>
+      </c>
+      <c r="D14" t="s">
         <v>45</v>
-      </c>
-      <c r="D14" t="s">
-        <v>46</v>
       </c>
       <c r="E14" t="s">
         <v>14</v>
@@ -1256,7 +1278,7 @@
         <v>120</v>
       </c>
       <c r="I14" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J14">
         <v>14760</v>
@@ -1264,13 +1286,13 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
+        <v>56</v>
+      </c>
+      <c r="B15" t="s">
         <v>57</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>58</v>
-      </c>
-      <c r="C15" t="s">
-        <v>59</v>
       </c>
       <c r="D15" t="s">
         <v>13</v>
@@ -1296,16 +1318,16 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
+        <v>59</v>
+      </c>
+      <c r="B16" t="s">
         <v>60</v>
       </c>
-      <c r="B16" t="s">
-        <v>61</v>
-      </c>
       <c r="C16" t="s">
+        <v>48</v>
+      </c>
+      <c r="D16" t="s">
         <v>49</v>
-      </c>
-      <c r="D16" t="s">
-        <v>50</v>
       </c>
       <c r="E16" t="s">
         <v>14</v>
@@ -1328,16 +1350,16 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
+        <v>61</v>
+      </c>
+      <c r="B17" t="s">
         <v>62</v>
       </c>
-      <c r="B17" t="s">
-        <v>63</v>
-      </c>
       <c r="C17" t="s">
+        <v>48</v>
+      </c>
+      <c r="D17" t="s">
         <v>49</v>
-      </c>
-      <c r="D17" t="s">
-        <v>50</v>
       </c>
       <c r="E17" t="s">
         <v>14</v>
@@ -1352,7 +1374,7 @@
         <v>800</v>
       </c>
       <c r="I17" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J17">
         <v>136800</v>
@@ -1360,7 +1382,7 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B18" t="s">
         <v>11</v>
@@ -1392,16 +1414,16 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
+        <v>64</v>
+      </c>
+      <c r="B19" t="s">
         <v>65</v>
       </c>
-      <c r="B19" t="s">
-        <v>66</v>
-      </c>
       <c r="C19" t="s">
+        <v>34</v>
+      </c>
+      <c r="D19" t="s">
         <v>35</v>
-      </c>
-      <c r="D19" t="s">
-        <v>36</v>
       </c>
       <c r="E19" t="s">
         <v>14</v>
@@ -1410,13 +1432,13 @@
         <v>1965</v>
       </c>
       <c r="G19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H19">
         <v>120</v>
       </c>
       <c r="I19" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J19">
         <v>21360</v>
@@ -1424,16 +1446,16 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
+        <v>66</v>
+      </c>
+      <c r="B20" t="s">
         <v>67</v>
       </c>
-      <c r="B20" t="s">
-        <v>68</v>
-      </c>
       <c r="C20" t="s">
+        <v>48</v>
+      </c>
+      <c r="D20" t="s">
         <v>49</v>
-      </c>
-      <c r="D20" t="s">
-        <v>50</v>
       </c>
       <c r="E20" t="s">
         <v>14</v>
@@ -1442,13 +1464,13 @@
         <v>2015</v>
       </c>
       <c r="G20" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H20">
         <v>800</v>
       </c>
       <c r="I20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J20">
         <v>114400</v>
@@ -1456,16 +1478,16 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
+        <v>68</v>
+      </c>
+      <c r="B21" t="s">
         <v>69</v>
       </c>
-      <c r="B21" t="s">
-        <v>70</v>
-      </c>
       <c r="C21" t="s">
+        <v>19</v>
+      </c>
+      <c r="D21" t="s">
         <v>20</v>
-      </c>
-      <c r="D21" t="s">
-        <v>21</v>
       </c>
       <c r="E21" t="s">
         <v>14</v>
@@ -1474,13 +1496,13 @@
         <v>1995</v>
       </c>
       <c r="G21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H21">
         <v>1200</v>
       </c>
       <c r="I21" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J21">
         <v>116400</v>
@@ -1488,16 +1510,16 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
+        <v>70</v>
+      </c>
+      <c r="B22" t="s">
         <v>71</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D22" t="s">
         <v>72</v>
-      </c>
-      <c r="C22" t="s">
-        <v>25</v>
-      </c>
-      <c r="D22" t="s">
-        <v>73</v>
       </c>
       <c r="E22" t="s">
         <v>14</v>
@@ -1506,13 +1528,13 @@
         <v>2005</v>
       </c>
       <c r="G22" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H22">
         <v>2500</v>
       </c>
       <c r="I22" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J22">
         <v>312500</v>
@@ -1520,16 +1542,16 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
+        <v>73</v>
+      </c>
+      <c r="B23" t="s">
         <v>74</v>
       </c>
-      <c r="B23" t="s">
-        <v>75</v>
-      </c>
       <c r="C23" t="s">
+        <v>24</v>
+      </c>
+      <c r="D23" t="s">
         <v>25</v>
-      </c>
-      <c r="D23" t="s">
-        <v>26</v>
       </c>
       <c r="E23" t="s">
         <v>14</v>
@@ -1538,13 +1560,13 @@
         <v>1975</v>
       </c>
       <c r="G23" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H23">
         <v>250</v>
       </c>
       <c r="I23" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J23">
         <v>27250</v>
@@ -1552,16 +1574,16 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
+        <v>75</v>
+      </c>
+      <c r="B24" t="s">
         <v>76</v>
       </c>
-      <c r="B24" t="s">
-        <v>77</v>
-      </c>
       <c r="C24" t="s">
+        <v>40</v>
+      </c>
+      <c r="D24" t="s">
         <v>41</v>
-      </c>
-      <c r="D24" t="s">
-        <v>42</v>
       </c>
       <c r="E24" t="s">
         <v>14</v>
@@ -1576,7 +1598,7 @@
         <v>250</v>
       </c>
       <c r="I24" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J24">
         <v>29000</v>
@@ -1584,16 +1606,16 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
+        <v>77</v>
+      </c>
+      <c r="B25" t="s">
         <v>78</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
+        <v>19</v>
+      </c>
+      <c r="D25" t="s">
         <v>79</v>
-      </c>
-      <c r="C25" t="s">
-        <v>20</v>
-      </c>
-      <c r="D25" t="s">
-        <v>80</v>
       </c>
       <c r="E25" t="s">
         <v>14</v>
@@ -1608,21 +1630,21 @@
         <v>400</v>
       </c>
       <c r="I25" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
+        <v>80</v>
+      </c>
+      <c r="B26" t="s">
         <v>81</v>
       </c>
-      <c r="B26" t="s">
-        <v>82</v>
-      </c>
       <c r="C26" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D26" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E26" t="s">
         <v>14</v>
@@ -1637,7 +1659,7 @@
         <v>800</v>
       </c>
       <c r="I26" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J26">
         <v>104800</v>
@@ -1645,16 +1667,16 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
+        <v>82</v>
+      </c>
+      <c r="B27" t="s">
         <v>83</v>
       </c>
-      <c r="B27" t="s">
-        <v>84</v>
-      </c>
       <c r="C27" t="s">
+        <v>24</v>
+      </c>
+      <c r="D27" t="s">
         <v>25</v>
-      </c>
-      <c r="D27" t="s">
-        <v>26</v>
       </c>
       <c r="E27" t="s">
         <v>14</v>
@@ -1677,16 +1699,16 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
+        <v>84</v>
+      </c>
+      <c r="B28" t="s">
         <v>85</v>
       </c>
-      <c r="B28" t="s">
-        <v>86</v>
-      </c>
       <c r="C28" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" t="s">
         <v>20</v>
-      </c>
-      <c r="D28" t="s">
-        <v>21</v>
       </c>
       <c r="E28" t="s">
         <v>14</v>
@@ -1695,13 +1717,13 @@
         <v>1995</v>
       </c>
       <c r="G28" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H28">
         <v>120</v>
       </c>
       <c r="I28" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J28">
         <v>18720</v>
@@ -1709,16 +1731,16 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
+        <v>86</v>
+      </c>
+      <c r="B29" t="s">
         <v>87</v>
       </c>
-      <c r="B29" t="s">
-        <v>88</v>
-      </c>
       <c r="C29" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D29" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E29" t="s">
         <v>14</v>
@@ -1741,16 +1763,16 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
+        <v>88</v>
+      </c>
+      <c r="B30" t="s">
         <v>89</v>
       </c>
-      <c r="B30" t="s">
-        <v>90</v>
-      </c>
       <c r="C30" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D30" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E30" t="s">
         <v>14</v>
@@ -1765,7 +1787,7 @@
         <v>800</v>
       </c>
       <c r="I30" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J30">
         <v>9999999</v>
@@ -1773,16 +1795,16 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
+        <v>90</v>
+      </c>
+      <c r="B31" t="s">
         <v>91</v>
       </c>
-      <c r="B31" t="s">
-        <v>92</v>
-      </c>
       <c r="C31" t="s">
+        <v>48</v>
+      </c>
+      <c r="D31" t="s">
         <v>49</v>
-      </c>
-      <c r="D31" t="s">
-        <v>50</v>
       </c>
       <c r="E31" t="s">
         <v>14</v>
@@ -1791,7 +1813,7 @@
         <v>2005</v>
       </c>
       <c r="G31" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H31">
         <v>800</v>
@@ -1805,16 +1827,16 @@
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
+        <v>92</v>
+      </c>
+      <c r="B32" t="s">
         <v>93</v>
       </c>
-      <c r="B32" t="s">
-        <v>94</v>
-      </c>
       <c r="C32" t="s">
+        <v>44</v>
+      </c>
+      <c r="D32" t="s">
         <v>45</v>
-      </c>
-      <c r="D32" t="s">
-        <v>46</v>
       </c>
       <c r="E32" t="s">
         <v>14</v>
@@ -1823,7 +1845,7 @@
         <v>1995</v>
       </c>
       <c r="G32" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H32">
         <v>400</v>
@@ -1837,16 +1859,16 @@
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
+        <v>94</v>
+      </c>
+      <c r="B33" t="s">
         <v>95</v>
       </c>
-      <c r="B33" t="s">
-        <v>96</v>
-      </c>
       <c r="C33" t="s">
+        <v>19</v>
+      </c>
+      <c r="D33" t="s">
         <v>20</v>
-      </c>
-      <c r="D33" t="s">
-        <v>21</v>
       </c>
       <c r="E33" t="s">
         <v>14</v>
@@ -1861,7 +1883,7 @@
         <v>400</v>
       </c>
       <c r="I33" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J33">
         <v>67200</v>
@@ -1869,16 +1891,16 @@
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>96</v>
+      </c>
+      <c r="B34" t="s">
         <v>97</v>
       </c>
-      <c r="B34" t="s">
-        <v>98</v>
-      </c>
       <c r="C34" t="s">
+        <v>34</v>
+      </c>
+      <c r="D34" t="s">
         <v>35</v>
-      </c>
-      <c r="D34" t="s">
-        <v>36</v>
       </c>
       <c r="E34" t="s">
         <v>14</v>
@@ -1887,13 +1909,13 @@
         <v>1965</v>
       </c>
       <c r="G34" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H34">
         <v>1200</v>
       </c>
       <c r="I34" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J34">
         <v>117600</v>
@@ -1901,16 +1923,16 @@
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
+        <v>98</v>
+      </c>
+      <c r="B35" t="s">
         <v>99</v>
       </c>
-      <c r="B35" t="s">
-        <v>100</v>
-      </c>
       <c r="C35" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D35" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E35" t="s">
         <v>14</v>
@@ -1919,7 +1941,7 @@
         <v>2005</v>
       </c>
       <c r="G35" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H35">
         <v>2500</v>
@@ -1933,16 +1955,16 @@
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
+        <v>100</v>
+      </c>
+      <c r="B36" t="s">
         <v>101</v>
       </c>
-      <c r="B36" t="s">
-        <v>102</v>
-      </c>
       <c r="C36" t="s">
+        <v>48</v>
+      </c>
+      <c r="D36" t="s">
         <v>49</v>
-      </c>
-      <c r="D36" t="s">
-        <v>50</v>
       </c>
       <c r="E36" t="s">
         <v>14</v>
@@ -1951,13 +1973,13 @@
         <v>1985</v>
       </c>
       <c r="G36" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H36">
         <v>400</v>
       </c>
       <c r="I36" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J36">
         <v>59200</v>
@@ -1965,10 +1987,10 @@
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
+        <v>102</v>
+      </c>
+      <c r="B37" t="s">
         <v>103</v>
-      </c>
-      <c r="B37" t="s">
-        <v>104</v>
       </c>
       <c r="C37" t="s">
         <v>12</v>
@@ -1989,7 +2011,7 @@
         <v>250</v>
       </c>
       <c r="I37" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J37">
         <v>32750</v>
@@ -1997,16 +2019,16 @@
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
+        <v>104</v>
+      </c>
+      <c r="B38" t="s">
         <v>105</v>
       </c>
-      <c r="B38" t="s">
-        <v>106</v>
-      </c>
       <c r="C38" t="s">
+        <v>40</v>
+      </c>
+      <c r="D38" t="s">
         <v>41</v>
-      </c>
-      <c r="D38" t="s">
-        <v>42</v>
       </c>
       <c r="E38" t="s">
         <v>14</v>
@@ -2015,7 +2037,7 @@
         <v>2005</v>
       </c>
       <c r="G38" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H38">
         <v>400</v>
@@ -2029,16 +2051,16 @@
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B39" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C39" t="s">
+        <v>48</v>
+      </c>
+      <c r="D39" t="s">
         <v>49</v>
-      </c>
-      <c r="D39" t="s">
-        <v>50</v>
       </c>
       <c r="E39" t="s">
         <v>14</v>
@@ -2047,13 +2069,13 @@
         <v>1985</v>
       </c>
       <c r="G39" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H39">
         <v>2500</v>
       </c>
       <c r="I39" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J39">
         <v>342500</v>
@@ -2061,10 +2083,10 @@
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
+        <v>107</v>
+      </c>
+      <c r="B40" t="s">
         <v>108</v>
-      </c>
-      <c r="B40" t="s">
-        <v>109</v>
       </c>
       <c r="C40" t="s">
         <v>12</v>
@@ -2076,13 +2098,13 @@
         <v>1965</v>
       </c>
       <c r="G40" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H40">
         <v>120</v>
       </c>
       <c r="I40" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J40">
         <v>16800</v>
@@ -2090,16 +2112,16 @@
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
+        <v>109</v>
+      </c>
+      <c r="B41" t="s">
         <v>110</v>
       </c>
-      <c r="B41" t="s">
-        <v>111</v>
-      </c>
       <c r="C41" t="s">
+        <v>40</v>
+      </c>
+      <c r="D41" t="s">
         <v>41</v>
-      </c>
-      <c r="D41" t="s">
-        <v>42</v>
       </c>
       <c r="E41" t="s">
         <v>14</v>
@@ -2108,7 +2130,7 @@
         <v>1975</v>
       </c>
       <c r="G41" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H41">
         <v>1200</v>
@@ -2122,10 +2144,10 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
+        <v>111</v>
+      </c>
+      <c r="B42" t="s">
         <v>112</v>
-      </c>
-      <c r="B42" t="s">
-        <v>113</v>
       </c>
       <c r="C42" t="s">
         <v>12</v>
@@ -2140,7 +2162,7 @@
         <v>2015</v>
       </c>
       <c r="G42" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H42">
         <v>2500</v>
@@ -2154,16 +2176,16 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
+        <v>113</v>
+      </c>
+      <c r="B43" t="s">
         <v>114</v>
       </c>
-      <c r="B43" t="s">
-        <v>115</v>
-      </c>
       <c r="C43" t="s">
+        <v>40</v>
+      </c>
+      <c r="D43" t="s">
         <v>41</v>
-      </c>
-      <c r="D43" t="s">
-        <v>42</v>
       </c>
       <c r="E43" t="s">
         <v>14</v>
@@ -2172,13 +2194,13 @@
         <v>1975</v>
       </c>
       <c r="G43" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H43">
         <v>2500</v>
       </c>
       <c r="I43" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J43">
         <v>227500</v>
@@ -2186,16 +2208,16 @@
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
+        <v>115</v>
+      </c>
+      <c r="B44" t="s">
         <v>116</v>
       </c>
-      <c r="B44" t="s">
-        <v>117</v>
-      </c>
       <c r="C44" t="s">
+        <v>24</v>
+      </c>
+      <c r="D44" t="s">
         <v>25</v>
-      </c>
-      <c r="D44" t="s">
-        <v>26</v>
       </c>
       <c r="E44" t="s">
         <v>14</v>
@@ -2210,7 +2232,7 @@
         <v>120</v>
       </c>
       <c r="I44" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J44">
         <v>12120</v>
@@ -2218,16 +2240,16 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
+        <v>117</v>
+      </c>
+      <c r="B45" t="s">
         <v>118</v>
       </c>
-      <c r="B45" t="s">
-        <v>119</v>
-      </c>
       <c r="C45" t="s">
+        <v>34</v>
+      </c>
+      <c r="D45" t="s">
         <v>35</v>
-      </c>
-      <c r="D45" t="s">
-        <v>36</v>
       </c>
       <c r="E45" t="s">
         <v>14</v>
@@ -2242,7 +2264,7 @@
         <v>800</v>
       </c>
       <c r="I45" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J45">
         <v>126400</v>
@@ -2250,16 +2272,16 @@
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
+        <v>119</v>
+      </c>
+      <c r="B46" t="s">
         <v>120</v>
       </c>
-      <c r="B46" t="s">
-        <v>121</v>
-      </c>
       <c r="C46" t="s">
+        <v>44</v>
+      </c>
+      <c r="D46" t="s">
         <v>45</v>
-      </c>
-      <c r="D46" t="s">
-        <v>46</v>
       </c>
       <c r="E46" t="s">
         <v>14</v>
@@ -2268,13 +2290,13 @@
         <v>1985</v>
       </c>
       <c r="G46" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H46">
         <v>1200</v>
       </c>
       <c r="I46" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J46">
         <v>98400</v>
@@ -2282,16 +2304,16 @@
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
+        <v>121</v>
+      </c>
+      <c r="B47" t="s">
         <v>122</v>
       </c>
-      <c r="B47" t="s">
-        <v>123</v>
-      </c>
       <c r="C47" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D47" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E47" t="s">
         <v>14</v>
@@ -2306,7 +2328,7 @@
         <v>120</v>
       </c>
       <c r="I47" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J47">
         <v>16200</v>
@@ -2314,16 +2336,16 @@
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
+        <v>123</v>
+      </c>
+      <c r="B48" t="s">
         <v>124</v>
       </c>
-      <c r="B48" t="s">
-        <v>125</v>
-      </c>
       <c r="C48" t="s">
+        <v>40</v>
+      </c>
+      <c r="D48" t="s">
         <v>41</v>
-      </c>
-      <c r="D48" t="s">
-        <v>42</v>
       </c>
       <c r="E48" t="s">
         <v>14</v>
@@ -2332,13 +2354,13 @@
         <v>1975</v>
       </c>
       <c r="G48" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H48">
         <v>400</v>
       </c>
       <c r="I48" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J48">
         <v>46800</v>
@@ -2346,16 +2368,16 @@
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
+        <v>125</v>
+      </c>
+      <c r="B49" t="s">
         <v>126</v>
       </c>
-      <c r="B49" t="s">
-        <v>127</v>
-      </c>
       <c r="C49" t="s">
+        <v>40</v>
+      </c>
+      <c r="D49" t="s">
         <v>41</v>
-      </c>
-      <c r="D49" t="s">
-        <v>42</v>
       </c>
       <c r="E49" t="s">
         <v>14</v>
@@ -2364,13 +2386,13 @@
         <v>2005</v>
       </c>
       <c r="G49" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H49">
         <v>400</v>
       </c>
       <c r="I49" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J49">
         <v>38400</v>
@@ -2378,16 +2400,16 @@
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
+        <v>127</v>
+      </c>
+      <c r="B50" t="s">
         <v>128</v>
       </c>
-      <c r="B50" t="s">
-        <v>129</v>
-      </c>
       <c r="C50" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D50" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E50" t="s">
         <v>14</v>
@@ -2396,13 +2418,13 @@
         <v>2015</v>
       </c>
       <c r="G50" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H50">
         <v>800</v>
       </c>
       <c r="I50" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J50">
         <v>115200</v>
@@ -2410,16 +2432,16 @@
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
+        <v>129</v>
+      </c>
+      <c r="B51" t="s">
         <v>130</v>
       </c>
-      <c r="B51" t="s">
-        <v>131</v>
-      </c>
       <c r="C51" t="s">
+        <v>34</v>
+      </c>
+      <c r="D51" t="s">
         <v>35</v>
-      </c>
-      <c r="D51" t="s">
-        <v>36</v>
       </c>
       <c r="E51" t="s">
         <v>14</v>

</xml_diff>

<commit_message>
feat: implement dynamic mapping for advanced TABULA energy and CO2 scenarios
</commit_message>
<xml_diff>
--- a/data/raw/building_data.xlsx
+++ b/data/raw/building_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ehska\Projects\building-data-pipeline\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F635BAD2-A558-4A6C-8774-25546DF83666}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B09001B2-50D9-4F04-A0EF-4395FC260F9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="building_data" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="144">
   <si>
     <t>Building_ID</t>
   </si>
@@ -448,6 +448,15 @@
   </si>
   <si>
     <t>District</t>
+  </si>
+  <si>
+    <t>AB</t>
+  </si>
+  <si>
+    <t>MFH</t>
+  </si>
+  <si>
+    <t>SFH</t>
   </si>
 </sst>
 </file>
@@ -861,7 +870,7 @@
         <v>2000</v>
       </c>
       <c r="G2" t="s">
-        <v>21</v>
+        <v>141</v>
       </c>
       <c r="H2">
         <v>25000</v>
@@ -896,10 +905,10 @@
         <v>14</v>
       </c>
       <c r="F3">
-        <v>2013</v>
+        <v>1985</v>
       </c>
       <c r="G3" t="s">
-        <v>21</v>
+        <v>142</v>
       </c>
       <c r="H3">
         <v>100000</v>
@@ -934,10 +943,10 @@
         <v>14</v>
       </c>
       <c r="F4">
-        <v>1160</v>
+        <v>1915</v>
       </c>
       <c r="G4" t="s">
-        <v>15</v>
+        <v>143</v>
       </c>
       <c r="H4">
         <v>3500</v>

</xml_diff>